<commit_message>
MIN-based margin tiers; hide actual margin in output, add Margin Tier and Commission %
</commit_message>
<xml_diff>
--- a/rates.xlsx
+++ b/rates.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,14 +27,10 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="00666666"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -70,18 +66,19 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,100 +445,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>อัตรา Incentive ตาม Type และ Margin</t>
+          <t>TYPE/MARGIN</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>กรอกเฉพาะช่องสีเหลือง</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>กรอกเฉพาะช่องสีเหลือง  •  Margin ตั้งแต่ (≥) / น้อยกว่า (&lt;) กรอกเป็น %  •  เว้นว่างช่วงล่างสุด/บนสุด = ไม่จำกัด</t>
+          <t>OCOP</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Tier = MIN สูงสุดที่ Margin ถึง (Margin ≥ MIN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>OCNP</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Margin ต่ำกว่า MIN ของ Tier ต่ำสุด = ไม่ได้ Commission</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TYPE/MARGIN</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>&lt; 20%</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>20-40%</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>&gt;40%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Margin ตั้งแต่ (≥)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Margin น้อยกว่า (&lt;)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>MARGIN TYPE</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>OCOP</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>OCNP</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>

</xml_diff>